<commit_message>
data(reference): update reference data
</commit_message>
<xml_diff>
--- a/data/reference/raw_ref.xlsx
+++ b/data/reference/raw_ref.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Downloads\food-delivery-etl-dwh\data\reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC41E203-A12B-4920-80A5-C14EF1F7952F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2F5F312-D20D-4F71-9904-2485DE82A4A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1837" yWindow="1837" windowWidth="14401" windowHeight="8723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_ref_city" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="167">
   <si>
     <t>city_code</t>
   </si>
@@ -534,6 +534,12 @@
   </si>
   <si>
     <t>EV CYCLE</t>
+  </si>
+  <si>
+    <t>Delhi</t>
+  </si>
+  <si>
+    <t>DELHI</t>
   </si>
 </sst>
 </file>
@@ -574,7 +580,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -585,7 +591,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -650,8 +655,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ref_city" displayName="ref_city" ref="A1:C20" totalsRowShown="0">
-  <autoFilter ref="A1:C20" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ref_city" displayName="ref_city" ref="A1:C21" totalsRowShown="0">
+  <autoFilter ref="A1:C21" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="city_code"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="city_name"/>
@@ -1050,7 +1055,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="15.9375" customWidth="1"/>
@@ -1137,10 +1142,10 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>166</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>165</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -1148,10 +1153,10 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>5</v>
+        <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -1159,10 +1164,10 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -1170,10 +1175,10 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -1181,10 +1186,10 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B12" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C12">
         <v>1</v>
@@ -1192,10 +1197,10 @@
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="C13">
         <v>1</v>
@@ -1203,10 +1208,10 @@
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -1214,10 +1219,10 @@
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -1225,10 +1230,10 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="B16" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C16">
         <v>1</v>
@@ -1236,10 +1241,10 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="B17" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -1247,10 +1252,10 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>3</v>
+        <v>37</v>
       </c>
       <c r="B18" t="s">
-        <v>4</v>
+        <v>38</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -1258,10 +1263,10 @@
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -1269,12 +1274,23 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
+        <v>29</v>
+      </c>
+      <c r="B20" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" t="s">
         <v>35</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B21" t="s">
         <v>36</v>
       </c>
-      <c r="C20">
+      <c r="C21">
         <v>1</v>
       </c>
     </row>
@@ -1727,7 +1743,7 @@
       </c>
     </row>
     <row r="14" spans="1:3">
-      <c r="A14" s="4" t="s">
+      <c r="A14" t="s">
         <v>113</v>
       </c>
       <c r="B14" t="s">
@@ -1782,7 +1798,7 @@
       </c>
     </row>
     <row r="19" spans="1:3">
-      <c r="A19" s="4" t="s">
+      <c r="A19" t="s">
         <v>116</v>
       </c>
       <c r="B19" t="s">

</xml_diff>